<commit_message>
Deploying to gh-pages from  @ ea7092e266eb3ea3a43bea825bbd83b20d11f882 🚀
</commit_message>
<xml_diff>
--- a/assets/excel/2026_1-2-3.xlsx
+++ b/assets/excel/2026_1-2-3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Hannover\Dez15_Uebergreifende_Analysen\Projekte\Integrationsmonitoring\Schlesier\MT_Site\assets\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ACE5E9C-6F97-4CF9-BC21-687093D8F795}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9506499-64A9-4421-BDD4-2B0CE2D3F385}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{7A2C9C5F-6188-4B6C-9270-BAA72B6F2974}"/>
   </bookViews>
@@ -435,13 +435,13 @@
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -794,50 +794,50 @@
       </c>
     </row>
     <row r="6" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D6" s="17" t="s">
+      <c r="D6" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="E6" s="18" t="s">
+      <c r="E6" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="F6" s="18" t="s">
+      <c r="F6" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="G6" s="18" t="s">
+      <c r="G6" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="H6" s="18"/>
-      <c r="I6" s="18"/>
-      <c r="J6" s="18"/>
-      <c r="K6" s="18"/>
-      <c r="L6" s="18"/>
-      <c r="M6" s="18" t="s">
+      <c r="H6" s="17"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="17"/>
+      <c r="K6" s="17"/>
+      <c r="L6" s="17"/>
+      <c r="M6" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="N6" s="18" t="s">
+      <c r="N6" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="O6" s="18"/>
-      <c r="P6" s="18"/>
-      <c r="Q6" s="18"/>
-      <c r="R6" s="18"/>
-      <c r="S6" s="18"/>
-      <c r="T6" s="18" t="s">
+      <c r="O6" s="17"/>
+      <c r="P6" s="17"/>
+      <c r="Q6" s="17"/>
+      <c r="R6" s="17"/>
+      <c r="S6" s="17"/>
+      <c r="T6" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="U6" s="18" t="s">
+      <c r="U6" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="V6" s="18"/>
-      <c r="W6" s="18"/>
-      <c r="X6" s="18"/>
-      <c r="Y6" s="18"/>
-      <c r="Z6" s="19"/>
+      <c r="V6" s="17"/>
+      <c r="W6" s="17"/>
+      <c r="X6" s="17"/>
+      <c r="Y6" s="17"/>
+      <c r="Z6" s="18"/>
     </row>
     <row r="7" spans="2:26" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="D7" s="17"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="17"/>
+      <c r="F7" s="17"/>
       <c r="G7" s="3" t="s">
         <v>10</v>
       </c>
@@ -856,7 +856,7 @@
       <c r="L7" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="M7" s="18"/>
+      <c r="M7" s="17"/>
       <c r="N7" s="3" t="s">
         <v>10</v>
       </c>
@@ -875,7 +875,7 @@
       <c r="S7" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="T7" s="18"/>
+      <c r="T7" s="17"/>
       <c r="U7" s="3" t="s">
         <v>10</v>
       </c>
@@ -902,35 +902,35 @@
       <c r="C8" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="17"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18" t="s">
+      <c r="D8" s="19"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="18"/>
-      <c r="H8" s="18"/>
-      <c r="I8" s="18"/>
-      <c r="J8" s="18"/>
-      <c r="K8" s="18"/>
-      <c r="L8" s="18"/>
-      <c r="M8" s="18" t="s">
+      <c r="G8" s="17"/>
+      <c r="H8" s="17"/>
+      <c r="I8" s="17"/>
+      <c r="J8" s="17"/>
+      <c r="K8" s="17"/>
+      <c r="L8" s="17"/>
+      <c r="M8" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="N8" s="18"/>
-      <c r="O8" s="18"/>
-      <c r="P8" s="18"/>
-      <c r="Q8" s="18"/>
-      <c r="R8" s="18"/>
-      <c r="S8" s="18"/>
-      <c r="T8" s="18" t="s">
+      <c r="N8" s="17"/>
+      <c r="O8" s="17"/>
+      <c r="P8" s="17"/>
+      <c r="Q8" s="17"/>
+      <c r="R8" s="17"/>
+      <c r="S8" s="17"/>
+      <c r="T8" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="U8" s="18"/>
-      <c r="V8" s="18"/>
-      <c r="W8" s="18"/>
-      <c r="X8" s="18"/>
-      <c r="Y8" s="18"/>
-      <c r="Z8" s="19"/>
+      <c r="U8" s="17"/>
+      <c r="V8" s="17"/>
+      <c r="W8" s="17"/>
+      <c r="X8" s="17"/>
+      <c r="Y8" s="17"/>
+      <c r="Z8" s="18"/>
     </row>
     <row r="9" spans="2:26" s="11" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="C9" s="11">
@@ -943,7 +943,7 @@
         <v>2025</v>
       </c>
       <c r="F9" s="11">
-        <v>36370</v>
+        <v>36735</v>
       </c>
       <c r="G9" s="11">
         <v>2320</v>
@@ -964,7 +964,7 @@
         <v>15375</v>
       </c>
       <c r="M9" s="11">
-        <v>18770</v>
+        <v>18920</v>
       </c>
       <c r="N9" s="11">
         <v>1255</v>
@@ -985,7 +985,7 @@
         <v>7870</v>
       </c>
       <c r="T9" s="11">
-        <v>17600</v>
+        <v>17815</v>
       </c>
       <c r="U9" s="11">
         <v>1070</v>
@@ -1017,7 +1017,7 @@
         <v>2025</v>
       </c>
       <c r="F10" s="11">
-        <v>25170</v>
+        <v>25090</v>
       </c>
       <c r="G10" s="11">
         <v>1095</v>
@@ -1038,7 +1038,7 @@
         <v>11415</v>
       </c>
       <c r="M10" s="11">
-        <v>13510</v>
+        <v>13515</v>
       </c>
       <c r="N10" s="11">
         <v>655</v>
@@ -1059,7 +1059,7 @@
         <v>6120</v>
       </c>
       <c r="T10" s="11">
-        <v>11650</v>
+        <v>11575</v>
       </c>
       <c r="U10" s="11">
         <v>440</v>
@@ -1091,7 +1091,7 @@
         <v>2025</v>
       </c>
       <c r="F11" s="11">
-        <v>25945</v>
+        <v>26115</v>
       </c>
       <c r="G11" s="11">
         <v>1470</v>
@@ -1112,7 +1112,7 @@
         <v>11290</v>
       </c>
       <c r="M11" s="11">
-        <v>13595</v>
+        <v>13710</v>
       </c>
       <c r="N11" s="11">
         <v>820</v>
@@ -1133,7 +1133,7 @@
         <v>6050</v>
       </c>
       <c r="T11" s="11">
-        <v>12355</v>
+        <v>12405</v>
       </c>
       <c r="U11" s="11">
         <v>650</v>
@@ -1165,7 +1165,7 @@
         <v>2025</v>
       </c>
       <c r="F12" s="11">
-        <v>17880</v>
+        <v>17575</v>
       </c>
       <c r="G12" s="11">
         <v>940</v>
@@ -1186,7 +1186,7 @@
         <v>7505</v>
       </c>
       <c r="M12" s="11">
-        <v>9420</v>
+        <v>9125</v>
       </c>
       <c r="N12" s="11">
         <v>475</v>
@@ -1207,7 +1207,7 @@
         <v>3835</v>
       </c>
       <c r="T12" s="11">
-        <v>8460</v>
+        <v>8465</v>
       </c>
       <c r="U12" s="11">
         <v>465</v>
@@ -1239,7 +1239,7 @@
         <v>2025</v>
       </c>
       <c r="F13" s="11">
-        <v>17035</v>
+        <v>16155</v>
       </c>
       <c r="G13" s="11">
         <v>1480</v>
@@ -1260,7 +1260,7 @@
         <v>5485</v>
       </c>
       <c r="M13" s="11">
-        <v>9220</v>
+        <v>8580</v>
       </c>
       <c r="N13" s="11">
         <v>870</v>
@@ -1281,7 +1281,7 @@
         <v>2890</v>
       </c>
       <c r="T13" s="11">
-        <v>7810</v>
+        <v>7575</v>
       </c>
       <c r="U13" s="11">
         <v>610</v>
@@ -1313,7 +1313,7 @@
         <v>2025</v>
       </c>
       <c r="F14" s="11">
-        <v>9500</v>
+        <v>9700</v>
       </c>
       <c r="G14" s="11">
         <v>695</v>
@@ -1334,7 +1334,7 @@
         <v>3975</v>
       </c>
       <c r="M14" s="11">
-        <v>4935</v>
+        <v>5050</v>
       </c>
       <c r="N14" s="11">
         <v>395</v>
@@ -1355,7 +1355,7 @@
         <v>2155</v>
       </c>
       <c r="T14" s="11">
-        <v>4570</v>
+        <v>4645</v>
       </c>
       <c r="U14" s="11">
         <v>300</v>
@@ -1387,7 +1387,7 @@
         <v>2025</v>
       </c>
       <c r="F15" s="11">
-        <v>13980</v>
+        <v>13385</v>
       </c>
       <c r="G15" s="11">
         <v>610</v>
@@ -1408,7 +1408,7 @@
         <v>5110</v>
       </c>
       <c r="M15" s="11">
-        <v>7355</v>
+        <v>7020</v>
       </c>
       <c r="N15" s="11">
         <v>365</v>
@@ -1429,7 +1429,7 @@
         <v>2630</v>
       </c>
       <c r="T15" s="11">
-        <v>6625</v>
+        <v>6375</v>
       </c>
       <c r="U15" s="11">
         <v>250</v>
@@ -1461,7 +1461,7 @@
         <v>2025</v>
       </c>
       <c r="F16" s="11">
-        <v>16325</v>
+        <v>16480</v>
       </c>
       <c r="G16" s="11">
         <v>1000</v>
@@ -1482,7 +1482,7 @@
         <v>6955</v>
       </c>
       <c r="M16" s="11">
-        <v>8540</v>
+        <v>8665</v>
       </c>
       <c r="N16" s="11">
         <v>600</v>
@@ -1503,7 +1503,7 @@
         <v>3575</v>
       </c>
       <c r="T16" s="11">
-        <v>7790</v>
+        <v>7815</v>
       </c>
       <c r="U16" s="11">
         <v>395</v>
@@ -1535,7 +1535,7 @@
         <v>2025</v>
       </c>
       <c r="F17" s="11">
-        <v>11105</v>
+        <v>11175</v>
       </c>
       <c r="G17" s="11">
         <v>650</v>
@@ -1556,7 +1556,7 @@
         <v>4455</v>
       </c>
       <c r="M17" s="11">
-        <v>5900</v>
+        <v>5985</v>
       </c>
       <c r="N17" s="11">
         <v>400</v>
@@ -1577,7 +1577,7 @@
         <v>2340</v>
       </c>
       <c r="T17" s="11">
-        <v>5200</v>
+        <v>5180</v>
       </c>
       <c r="U17" s="11">
         <v>250</v>
@@ -1609,7 +1609,7 @@
         <v>2025</v>
       </c>
       <c r="F18" s="11">
-        <v>41480</v>
+        <v>42390</v>
       </c>
       <c r="G18" s="11">
         <v>3275</v>
@@ -1630,7 +1630,7 @@
         <v>15345</v>
       </c>
       <c r="M18" s="11">
-        <v>20950</v>
+        <v>21385</v>
       </c>
       <c r="N18" s="11">
         <v>1670</v>
@@ -1651,7 +1651,7 @@
         <v>7930</v>
       </c>
       <c r="T18" s="11">
-        <v>20525</v>
+        <v>21005</v>
       </c>
       <c r="U18" s="11">
         <v>1605</v>
@@ -1683,7 +1683,7 @@
         <v>2025</v>
       </c>
       <c r="F19" s="12">
-        <v>214780</v>
+        <v>214805</v>
       </c>
       <c r="G19" s="12">
         <v>13535</v>
@@ -1704,7 +1704,7 @@
         <v>86910</v>
       </c>
       <c r="M19" s="12">
-        <v>112205</v>
+        <v>111955</v>
       </c>
       <c r="N19" s="12">
         <v>7505</v>
@@ -1725,7 +1725,7 @@
         <v>45390</v>
       </c>
       <c r="T19" s="12">
-        <v>102575</v>
+        <v>102850</v>
       </c>
       <c r="U19" s="12">
         <v>6035</v>
@@ -1757,7 +1757,7 @@
         <v>2025</v>
       </c>
       <c r="F20" s="11">
-        <v>227495</v>
+        <v>225335</v>
       </c>
       <c r="G20" s="11">
         <v>8065</v>
@@ -1778,7 +1778,7 @@
         <v>111800</v>
       </c>
       <c r="M20" s="11">
-        <v>117655</v>
+        <v>116115</v>
       </c>
       <c r="N20" s="11">
         <v>4370</v>
@@ -1799,7 +1799,7 @@
         <v>57885</v>
       </c>
       <c r="T20" s="11">
-        <v>109840</v>
+        <v>109210</v>
       </c>
       <c r="U20" s="11">
         <v>3695</v>
@@ -1831,7 +1831,7 @@
         <v>2025</v>
       </c>
       <c r="F21" s="11">
-        <v>135030</v>
+        <v>130955</v>
       </c>
       <c r="G21" s="11">
         <v>3000</v>
@@ -1852,7 +1852,7 @@
         <v>65915</v>
       </c>
       <c r="M21" s="11">
-        <v>69770</v>
+        <v>66950</v>
       </c>
       <c r="N21" s="11">
         <v>1450</v>
@@ -1873,7 +1873,7 @@
         <v>33960</v>
       </c>
       <c r="T21" s="11">
-        <v>65260</v>
+        <v>64010</v>
       </c>
       <c r="U21" s="11">
         <v>1550</v>
@@ -1905,7 +1905,7 @@
         <v>2025</v>
       </c>
       <c r="F22" s="11">
-        <v>92465</v>
+        <v>94380</v>
       </c>
       <c r="G22" s="11">
         <v>5065</v>
@@ -1926,7 +1926,7 @@
         <v>45885</v>
       </c>
       <c r="M22" s="11">
-        <v>47885</v>
+        <v>49165</v>
       </c>
       <c r="N22" s="11">
         <v>2920</v>
@@ -1947,7 +1947,7 @@
         <v>23925</v>
       </c>
       <c r="T22" s="11">
-        <v>44580</v>
+        <v>45200</v>
       </c>
       <c r="U22" s="11">
         <v>2145</v>
@@ -1979,7 +1979,7 @@
         <v>2025</v>
       </c>
       <c r="F23" s="11">
-        <v>26125</v>
+        <v>25910</v>
       </c>
       <c r="G23" s="11">
         <v>1515</v>
@@ -2000,7 +2000,7 @@
         <v>10475</v>
       </c>
       <c r="M23" s="11">
-        <v>13415</v>
+        <v>13315</v>
       </c>
       <c r="N23" s="11">
         <v>845</v>
@@ -2021,7 +2021,7 @@
         <v>5435</v>
       </c>
       <c r="T23" s="11">
-        <v>12710</v>
+        <v>12600</v>
       </c>
       <c r="U23" s="11">
         <v>670</v>
@@ -2053,7 +2053,7 @@
         <v>2025</v>
       </c>
       <c r="F24" s="11">
-        <v>22250</v>
+        <v>22205</v>
       </c>
       <c r="G24" s="11">
         <v>935</v>
@@ -2074,7 +2074,7 @@
         <v>10500</v>
       </c>
       <c r="M24" s="11">
-        <v>11400</v>
+        <v>11355</v>
       </c>
       <c r="N24" s="11">
         <v>490</v>
@@ -2095,7 +2095,7 @@
         <v>5520</v>
       </c>
       <c r="T24" s="11">
-        <v>10850</v>
+        <v>10865</v>
       </c>
       <c r="U24" s="11">
         <v>445</v>
@@ -2127,7 +2127,7 @@
         <v>2025</v>
       </c>
       <c r="F25" s="11">
-        <v>33380</v>
+        <v>33590</v>
       </c>
       <c r="G25" s="11">
         <v>1885</v>
@@ -2148,7 +2148,7 @@
         <v>14020</v>
       </c>
       <c r="M25" s="11">
-        <v>17520</v>
+        <v>17665</v>
       </c>
       <c r="N25" s="11">
         <v>1045</v>
@@ -2169,7 +2169,7 @@
         <v>7335</v>
       </c>
       <c r="T25" s="11">
-        <v>15860</v>
+        <v>15925</v>
       </c>
       <c r="U25" s="11">
         <v>840</v>
@@ -2201,7 +2201,7 @@
         <v>2025</v>
       </c>
       <c r="F26" s="11">
-        <v>6910</v>
+        <v>6945</v>
       </c>
       <c r="G26" s="11">
         <v>310</v>
@@ -2222,7 +2222,7 @@
         <v>2760</v>
       </c>
       <c r="M26" s="11">
-        <v>3580</v>
+        <v>3570</v>
       </c>
       <c r="N26" s="11">
         <v>155</v>
@@ -2243,7 +2243,7 @@
         <v>1480</v>
       </c>
       <c r="T26" s="11">
-        <v>3340</v>
+        <v>3375</v>
       </c>
       <c r="U26" s="11">
         <v>160</v>
@@ -2275,7 +2275,7 @@
         <v>2025</v>
       </c>
       <c r="F27" s="11">
-        <v>14340</v>
+        <v>13945</v>
       </c>
       <c r="G27" s="11">
         <v>540</v>
@@ -2296,7 +2296,7 @@
         <v>5820</v>
       </c>
       <c r="M27" s="11">
-        <v>7445</v>
+        <v>7230</v>
       </c>
       <c r="N27" s="11">
         <v>290</v>
@@ -2317,7 +2317,7 @@
         <v>3105</v>
       </c>
       <c r="T27" s="11">
-        <v>6895</v>
+        <v>6725</v>
       </c>
       <c r="U27" s="11">
         <v>255</v>
@@ -2349,7 +2349,7 @@
         <v>2025</v>
       </c>
       <c r="F28" s="11">
-        <v>18950</v>
+        <v>18085</v>
       </c>
       <c r="G28" s="11">
         <v>895</v>
@@ -2370,7 +2370,7 @@
         <v>7925</v>
       </c>
       <c r="M28" s="11">
-        <v>9855</v>
+        <v>9385</v>
       </c>
       <c r="N28" s="11">
         <v>495</v>
@@ -2391,7 +2391,7 @@
         <v>4160</v>
       </c>
       <c r="T28" s="11">
-        <v>9095</v>
+        <v>8705</v>
       </c>
       <c r="U28" s="11">
         <v>405</v>
@@ -2423,7 +2423,7 @@
         <v>2025</v>
       </c>
       <c r="F29" s="12">
-        <v>349445</v>
+        <v>346025</v>
       </c>
       <c r="G29" s="12">
         <v>14145</v>
@@ -2444,7 +2444,7 @@
         <v>163300</v>
       </c>
       <c r="M29" s="12">
-        <v>180870</v>
+        <v>178625</v>
       </c>
       <c r="N29" s="12">
         <v>7685</v>
@@ -2465,7 +2465,7 @@
         <v>84915</v>
       </c>
       <c r="T29" s="12">
-        <v>168585</v>
+        <v>167395</v>
       </c>
       <c r="U29" s="12">
         <v>6460</v>
@@ -2497,7 +2497,7 @@
         <v>2025</v>
       </c>
       <c r="F30" s="11">
-        <v>18650</v>
+        <v>18760</v>
       </c>
       <c r="G30" s="11">
         <v>1035</v>
@@ -2518,7 +2518,7 @@
         <v>7930</v>
       </c>
       <c r="M30" s="11">
-        <v>9585</v>
+        <v>9580</v>
       </c>
       <c r="N30" s="11">
         <v>555</v>
@@ -2539,7 +2539,7 @@
         <v>4195</v>
       </c>
       <c r="T30" s="11">
-        <v>9075</v>
+        <v>9185</v>
       </c>
       <c r="U30" s="11">
         <v>480</v>
@@ -2571,7 +2571,7 @@
         <v>2025</v>
       </c>
       <c r="F31" s="11">
-        <v>17030</v>
+        <v>16890</v>
       </c>
       <c r="G31" s="11">
         <v>1005</v>
@@ -2592,7 +2592,7 @@
         <v>7510</v>
       </c>
       <c r="M31" s="11">
-        <v>8935</v>
+        <v>8865</v>
       </c>
       <c r="N31" s="11">
         <v>535</v>
@@ -2613,7 +2613,7 @@
         <v>3925</v>
       </c>
       <c r="T31" s="11">
-        <v>8090</v>
+        <v>8035</v>
       </c>
       <c r="U31" s="11">
         <v>470</v>
@@ -2645,7 +2645,7 @@
         <v>2025</v>
       </c>
       <c r="F32" s="11">
-        <v>31485</v>
+        <v>29810</v>
       </c>
       <c r="G32" s="11">
         <v>2070</v>
@@ -2666,7 +2666,7 @@
         <v>12220</v>
       </c>
       <c r="M32" s="11">
-        <v>18165</v>
+        <v>16930</v>
       </c>
       <c r="N32" s="11">
         <v>1200</v>
@@ -2687,7 +2687,7 @@
         <v>6695</v>
       </c>
       <c r="T32" s="11">
-        <v>13315</v>
+        <v>12875</v>
       </c>
       <c r="U32" s="11">
         <v>865</v>
@@ -2719,7 +2719,7 @@
         <v>2025</v>
       </c>
       <c r="F33" s="11">
-        <v>3920</v>
+        <v>3990</v>
       </c>
       <c r="G33" s="11">
         <v>360</v>
@@ -2740,7 +2740,7 @@
         <v>1405</v>
       </c>
       <c r="M33" s="11">
-        <v>1995</v>
+        <v>2060</v>
       </c>
       <c r="N33" s="11">
         <v>200</v>
@@ -2761,7 +2761,7 @@
         <v>750</v>
       </c>
       <c r="T33" s="11">
-        <v>1935</v>
+        <v>1930</v>
       </c>
       <c r="U33" s="11">
         <v>160</v>
@@ -2793,7 +2793,7 @@
         <v>2025</v>
       </c>
       <c r="F34" s="11">
-        <v>17600</v>
+        <v>17145</v>
       </c>
       <c r="G34" s="11">
         <v>1185</v>
@@ -2814,7 +2814,7 @@
         <v>6410</v>
       </c>
       <c r="M34" s="11">
-        <v>9065</v>
+        <v>8805</v>
       </c>
       <c r="N34" s="11">
         <v>575</v>
@@ -2835,7 +2835,7 @@
         <v>3460</v>
       </c>
       <c r="T34" s="11">
-        <v>8530</v>
+        <v>8340</v>
       </c>
       <c r="U34" s="11">
         <v>610</v>
@@ -2867,7 +2867,7 @@
         <v>2025</v>
       </c>
       <c r="F35" s="11">
-        <v>9375</v>
+        <v>9045</v>
       </c>
       <c r="G35" s="11">
         <v>430</v>
@@ -2888,7 +2888,7 @@
         <v>3920</v>
       </c>
       <c r="M35" s="11">
-        <v>4570</v>
+        <v>4410</v>
       </c>
       <c r="N35" s="11">
         <v>220</v>
@@ -2909,7 +2909,7 @@
         <v>1920</v>
       </c>
       <c r="T35" s="11">
-        <v>4810</v>
+        <v>4635</v>
       </c>
       <c r="U35" s="11">
         <v>210</v>
@@ -2941,7 +2941,7 @@
         <v>2025</v>
       </c>
       <c r="F36" s="11">
-        <v>16965</v>
+        <v>16880</v>
       </c>
       <c r="G36" s="11">
         <v>1150</v>
@@ -2962,7 +2962,7 @@
         <v>6350</v>
       </c>
       <c r="M36" s="11">
-        <v>9155</v>
+        <v>9170</v>
       </c>
       <c r="N36" s="11">
         <v>650</v>
@@ -2983,7 +2983,7 @@
         <v>3535</v>
       </c>
       <c r="T36" s="11">
-        <v>7810</v>
+        <v>7715</v>
       </c>
       <c r="U36" s="11">
         <v>500</v>
@@ -3015,7 +3015,7 @@
         <v>2025</v>
       </c>
       <c r="F37" s="11">
-        <v>15440</v>
+        <v>15170</v>
       </c>
       <c r="G37" s="11">
         <v>915</v>
@@ -3036,7 +3036,7 @@
         <v>5925</v>
       </c>
       <c r="M37" s="11">
-        <v>8005</v>
+        <v>7880</v>
       </c>
       <c r="N37" s="11">
         <v>525</v>
@@ -3057,7 +3057,7 @@
         <v>3110</v>
       </c>
       <c r="T37" s="11">
-        <v>7435</v>
+        <v>7300</v>
       </c>
       <c r="U37" s="11">
         <v>395</v>
@@ -3089,7 +3089,7 @@
         <v>2025</v>
       </c>
       <c r="F38" s="11">
-        <v>26815</v>
+        <v>26315</v>
       </c>
       <c r="G38" s="11">
         <v>1310</v>
@@ -3110,7 +3110,7 @@
         <v>10255</v>
       </c>
       <c r="M38" s="11">
-        <v>14360</v>
+        <v>14030</v>
       </c>
       <c r="N38" s="11">
         <v>695</v>
@@ -3131,7 +3131,7 @@
         <v>5645</v>
       </c>
       <c r="T38" s="11">
-        <v>12450</v>
+        <v>12285</v>
       </c>
       <c r="U38" s="11">
         <v>615</v>
@@ -3163,7 +3163,7 @@
         <v>2025</v>
       </c>
       <c r="F39" s="11">
-        <v>8145</v>
+        <v>8405</v>
       </c>
       <c r="G39" s="11">
         <v>635</v>
@@ -3184,7 +3184,7 @@
         <v>2995</v>
       </c>
       <c r="M39" s="11">
-        <v>4095</v>
+        <v>4235</v>
       </c>
       <c r="N39" s="11">
         <v>345</v>
@@ -3205,7 +3205,7 @@
         <v>1550</v>
       </c>
       <c r="T39" s="11">
-        <v>4050</v>
+        <v>4165</v>
       </c>
       <c r="U39" s="11">
         <v>290</v>
@@ -3237,7 +3237,7 @@
         <v>2025</v>
       </c>
       <c r="F40" s="11">
-        <v>15260</v>
+        <v>15550</v>
       </c>
       <c r="G40" s="11">
         <v>1030</v>
@@ -3258,7 +3258,7 @@
         <v>6660</v>
       </c>
       <c r="M40" s="11">
-        <v>8040</v>
+        <v>8200</v>
       </c>
       <c r="N40" s="11">
         <v>585</v>
@@ -3279,7 +3279,7 @@
         <v>3490</v>
       </c>
       <c r="T40" s="11">
-        <v>7225</v>
+        <v>7350</v>
       </c>
       <c r="U40" s="11">
         <v>445</v>
@@ -3311,7 +3311,7 @@
         <v>2025</v>
       </c>
       <c r="F41" s="12">
-        <v>180680</v>
+        <v>177980</v>
       </c>
       <c r="G41" s="12">
         <v>11125</v>
@@ -3332,7 +3332,7 @@
         <v>71580</v>
       </c>
       <c r="M41" s="12">
-        <v>95975</v>
+        <v>94155</v>
       </c>
       <c r="N41" s="12">
         <v>6080</v>
@@ -3353,7 +3353,7 @@
         <v>38275</v>
       </c>
       <c r="T41" s="12">
-        <v>84715</v>
+        <v>83815</v>
       </c>
       <c r="U41" s="12">
         <v>5045</v>
@@ -3385,7 +3385,7 @@
         <v>2025</v>
       </c>
       <c r="F42" s="11">
-        <v>16525</v>
+        <v>16415</v>
       </c>
       <c r="G42" s="11">
         <v>695</v>
@@ -3406,7 +3406,7 @@
         <v>7205</v>
       </c>
       <c r="M42" s="11">
-        <v>8400</v>
+        <v>8385</v>
       </c>
       <c r="N42" s="11">
         <v>385</v>
@@ -3427,7 +3427,7 @@
         <v>3765</v>
       </c>
       <c r="T42" s="11">
-        <v>8130</v>
+        <v>8040</v>
       </c>
       <c r="U42" s="11">
         <v>310</v>
@@ -3459,7 +3459,7 @@
         <v>2025</v>
       </c>
       <c r="F43" s="11">
-        <v>7525</v>
+        <v>7460</v>
       </c>
       <c r="G43" s="11">
         <v>450</v>
@@ -3480,7 +3480,7 @@
         <v>2525</v>
       </c>
       <c r="M43" s="11">
-        <v>4140</v>
+        <v>4065</v>
       </c>
       <c r="N43" s="11">
         <v>250</v>
@@ -3501,7 +3501,7 @@
         <v>1420</v>
       </c>
       <c r="T43" s="11">
-        <v>3385</v>
+        <v>3390</v>
       </c>
       <c r="U43" s="11">
         <v>200</v>
@@ -3533,7 +3533,7 @@
         <v>2025</v>
       </c>
       <c r="F44" s="11">
-        <v>23895</v>
+        <v>24185</v>
       </c>
       <c r="G44" s="11">
         <v>1380</v>
@@ -3554,7 +3554,7 @@
         <v>8985</v>
       </c>
       <c r="M44" s="11">
-        <v>11930</v>
+        <v>12140</v>
       </c>
       <c r="N44" s="11">
         <v>705</v>
@@ -3575,7 +3575,7 @@
         <v>4715</v>
       </c>
       <c r="T44" s="11">
-        <v>11970</v>
+        <v>12035</v>
       </c>
       <c r="U44" s="11">
         <v>675</v>
@@ -3607,7 +3607,7 @@
         <v>2025</v>
       </c>
       <c r="F45" s="11">
-        <v>31200</v>
+        <v>31870</v>
       </c>
       <c r="G45" s="11">
         <v>1450</v>
@@ -3628,7 +3628,7 @@
         <v>13515</v>
       </c>
       <c r="M45" s="11">
-        <v>16005</v>
+        <v>16350</v>
       </c>
       <c r="N45" s="11">
         <v>710</v>
@@ -3649,7 +3649,7 @@
         <v>7035</v>
       </c>
       <c r="T45" s="11">
-        <v>15195</v>
+        <v>15525</v>
       </c>
       <c r="U45" s="11">
         <v>740</v>
@@ -3681,7 +3681,7 @@
         <v>2025</v>
       </c>
       <c r="F46" s="11">
-        <v>12155</v>
+        <v>12035</v>
       </c>
       <c r="G46" s="11">
         <v>955</v>
@@ -3702,7 +3702,7 @@
         <v>4150</v>
       </c>
       <c r="M46" s="11">
-        <v>6680</v>
+        <v>6580</v>
       </c>
       <c r="N46" s="11">
         <v>545</v>
@@ -3755,7 +3755,7 @@
         <v>2025</v>
       </c>
       <c r="F47" s="11">
-        <v>11725</v>
+        <v>11890</v>
       </c>
       <c r="G47" s="11">
         <v>780</v>
@@ -3776,7 +3776,7 @@
         <v>4305</v>
       </c>
       <c r="M47" s="11">
-        <v>6145</v>
+        <v>6270</v>
       </c>
       <c r="N47" s="11">
         <v>450</v>
@@ -3797,7 +3797,7 @@
         <v>2300</v>
       </c>
       <c r="T47" s="11">
-        <v>5575</v>
+        <v>5620</v>
       </c>
       <c r="U47" s="11">
         <v>330</v>
@@ -3829,7 +3829,7 @@
         <v>2025</v>
       </c>
       <c r="F48" s="11">
-        <v>15580</v>
+        <v>15455</v>
       </c>
       <c r="G48" s="11">
         <v>1025</v>
@@ -3850,7 +3850,7 @@
         <v>5375</v>
       </c>
       <c r="M48" s="11">
-        <v>8555</v>
+        <v>8460</v>
       </c>
       <c r="N48" s="11">
         <v>555</v>
@@ -3871,7 +3871,7 @@
         <v>2980</v>
       </c>
       <c r="T48" s="11">
-        <v>7025</v>
+        <v>7000</v>
       </c>
       <c r="U48" s="11">
         <v>470</v>
@@ -3903,7 +3903,7 @@
         <v>2025</v>
       </c>
       <c r="F49" s="11">
-        <v>27545</v>
+        <v>26690</v>
       </c>
       <c r="G49" s="11">
         <v>1360</v>
@@ -3924,7 +3924,7 @@
         <v>9610</v>
       </c>
       <c r="M49" s="11">
-        <v>15145</v>
+        <v>14595</v>
       </c>
       <c r="N49" s="11">
         <v>790</v>
@@ -3945,7 +3945,7 @@
         <v>5425</v>
       </c>
       <c r="T49" s="11">
-        <v>12400</v>
+        <v>12095</v>
       </c>
       <c r="U49" s="11">
         <v>570</v>
@@ -3977,7 +3977,7 @@
         <v>2025</v>
       </c>
       <c r="F50" s="11">
-        <v>52605</v>
+        <v>52305</v>
       </c>
       <c r="G50" s="11">
         <v>3305</v>
@@ -3998,7 +3998,7 @@
         <v>19065</v>
       </c>
       <c r="M50" s="11">
-        <v>30030</v>
+        <v>29660</v>
       </c>
       <c r="N50" s="11">
         <v>1995</v>
@@ -4019,7 +4019,7 @@
         <v>11070</v>
       </c>
       <c r="T50" s="11">
-        <v>22575</v>
+        <v>22660</v>
       </c>
       <c r="U50" s="11">
         <v>1315</v>
@@ -4051,7 +4051,7 @@
         <v>2025</v>
       </c>
       <c r="F51" s="11">
-        <v>6945</v>
+        <v>6895</v>
       </c>
       <c r="G51" s="11">
         <v>390</v>
@@ -4072,7 +4072,7 @@
         <v>2695</v>
       </c>
       <c r="M51" s="11">
-        <v>3590</v>
+        <v>3525</v>
       </c>
       <c r="N51" s="11">
         <v>205</v>
@@ -4093,7 +4093,7 @@
         <v>1420</v>
       </c>
       <c r="T51" s="11">
-        <v>3365</v>
+        <v>3375</v>
       </c>
       <c r="U51" s="11">
         <v>190</v>
@@ -4125,7 +4125,7 @@
         <v>2025</v>
       </c>
       <c r="F52" s="11">
-        <v>26195</v>
+        <v>26535</v>
       </c>
       <c r="G52" s="11">
         <v>1465</v>
@@ -4146,7 +4146,7 @@
         <v>13075</v>
       </c>
       <c r="M52" s="11">
-        <v>14070</v>
+        <v>14235</v>
       </c>
       <c r="N52" s="11">
         <v>820</v>
@@ -4167,7 +4167,7 @@
         <v>7105</v>
       </c>
       <c r="T52" s="11">
-        <v>12130</v>
+        <v>12295</v>
       </c>
       <c r="U52" s="11">
         <v>645</v>
@@ -4199,7 +4199,7 @@
         <v>2025</v>
       </c>
       <c r="F53" s="11">
-        <v>19125</v>
+        <v>19105</v>
       </c>
       <c r="G53" s="11">
         <v>1195</v>
@@ -4220,7 +4220,7 @@
         <v>7375</v>
       </c>
       <c r="M53" s="11">
-        <v>10460</v>
+        <v>10375</v>
       </c>
       <c r="N53" s="11">
         <v>685</v>
@@ -4241,7 +4241,7 @@
         <v>4035</v>
       </c>
       <c r="T53" s="11">
-        <v>8660</v>
+        <v>8735</v>
       </c>
       <c r="U53" s="11">
         <v>510</v>
@@ -4273,7 +4273,7 @@
         <v>2025</v>
       </c>
       <c r="F54" s="11">
-        <v>15200</v>
+        <v>14895</v>
       </c>
       <c r="G54" s="11">
         <v>1175</v>
@@ -4294,7 +4294,7 @@
         <v>5330</v>
       </c>
       <c r="M54" s="11">
-        <v>8130</v>
+        <v>7950</v>
       </c>
       <c r="N54" s="11">
         <v>670</v>
@@ -4315,7 +4315,7 @@
         <v>2820</v>
       </c>
       <c r="T54" s="11">
-        <v>7080</v>
+        <v>6940</v>
       </c>
       <c r="U54" s="11">
         <v>505</v>
@@ -4347,7 +4347,7 @@
         <v>2025</v>
       </c>
       <c r="F55" s="11">
-        <v>42275</v>
+        <v>40995</v>
       </c>
       <c r="G55" s="11">
         <v>2575</v>
@@ -4368,7 +4368,7 @@
         <v>17075</v>
       </c>
       <c r="M55" s="11">
-        <v>22375</v>
+        <v>21670</v>
       </c>
       <c r="N55" s="11">
         <v>1450</v>
@@ -4389,7 +4389,7 @@
         <v>9055</v>
       </c>
       <c r="T55" s="11">
-        <v>19910</v>
+        <v>19330</v>
       </c>
       <c r="U55" s="11">
         <v>1125</v>
@@ -4421,7 +4421,7 @@
         <v>2025</v>
       </c>
       <c r="F56" s="11">
-        <v>24775</v>
+        <v>24025</v>
       </c>
       <c r="G56" s="11">
         <v>1620</v>
@@ -4442,7 +4442,7 @@
         <v>9990</v>
       </c>
       <c r="M56" s="11">
-        <v>13010</v>
+        <v>12665</v>
       </c>
       <c r="N56" s="11">
         <v>870</v>
@@ -4463,7 +4463,7 @@
         <v>5420</v>
       </c>
       <c r="T56" s="11">
-        <v>11775</v>
+        <v>11355</v>
       </c>
       <c r="U56" s="11">
         <v>755</v>
@@ -4495,7 +4495,7 @@
         <v>2025</v>
       </c>
       <c r="F57" s="11">
-        <v>10440</v>
+        <v>10800</v>
       </c>
       <c r="G57" s="11">
         <v>685</v>
@@ -4516,7 +4516,7 @@
         <v>4485</v>
       </c>
       <c r="M57" s="11">
-        <v>5645</v>
+        <v>5825</v>
       </c>
       <c r="N57" s="11">
         <v>395</v>
@@ -4537,7 +4537,7 @@
         <v>2435</v>
       </c>
       <c r="T57" s="11">
-        <v>4785</v>
+        <v>4975</v>
       </c>
       <c r="U57" s="11">
         <v>290</v>
@@ -4569,7 +4569,7 @@
         <v>2025</v>
       </c>
       <c r="F58" s="11">
-        <v>4475</v>
+        <v>4230</v>
       </c>
       <c r="G58" s="11">
         <v>265</v>
@@ -4590,7 +4590,7 @@
         <v>1285</v>
       </c>
       <c r="M58" s="11">
-        <v>2280</v>
+        <v>2125</v>
       </c>
       <c r="N58" s="11">
         <v>150</v>
@@ -4611,7 +4611,7 @@
         <v>660</v>
       </c>
       <c r="T58" s="11">
-        <v>2190</v>
+        <v>2110</v>
       </c>
       <c r="U58" s="11">
         <v>120</v>
@@ -4643,7 +4643,7 @@
         <v>2025</v>
       </c>
       <c r="F59" s="12">
-        <v>348190</v>
+        <v>345795</v>
       </c>
       <c r="G59" s="12">
         <v>20775</v>
@@ -4664,7 +4664,7 @@
         <v>136055</v>
       </c>
       <c r="M59" s="12">
-        <v>186575</v>
+        <v>184855</v>
       </c>
       <c r="N59" s="12">
         <v>11625</v>
@@ -4685,7 +4685,7 @@
         <v>74000</v>
       </c>
       <c r="T59" s="12">
-        <v>161600</v>
+        <v>160930</v>
       </c>
       <c r="U59" s="12">
         <v>9150</v>
@@ -4717,7 +4717,7 @@
         <v>2025</v>
       </c>
       <c r="F60" s="12">
-        <v>1093110</v>
+        <v>1084595</v>
       </c>
       <c r="G60" s="12">
         <v>59585</v>
@@ -4738,7 +4738,7 @@
         <v>457845</v>
       </c>
       <c r="M60" s="12">
-        <v>575625</v>
+        <v>569605</v>
       </c>
       <c r="N60" s="12">
         <v>32895</v>
@@ -4759,7 +4759,7 @@
         <v>242585</v>
       </c>
       <c r="T60" s="12">
-        <v>517485</v>
+        <v>514995</v>
       </c>
       <c r="U60" s="12">
         <v>26690</v>
@@ -88111,17 +88111,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="D6:D8"/>
+    <mergeCell ref="E6:E8"/>
+    <mergeCell ref="F6:F7"/>
+    <mergeCell ref="G6:L6"/>
+    <mergeCell ref="M6:M7"/>
     <mergeCell ref="T6:T7"/>
     <mergeCell ref="U6:Z6"/>
     <mergeCell ref="F8:L8"/>
     <mergeCell ref="M8:S8"/>
     <mergeCell ref="T8:Z8"/>
     <mergeCell ref="N6:S6"/>
-    <mergeCell ref="D6:D8"/>
-    <mergeCell ref="E6:E8"/>
-    <mergeCell ref="F6:F7"/>
-    <mergeCell ref="G6:L6"/>
-    <mergeCell ref="M6:M7"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="D1159" r:id="rId1" xr:uid="{A02DF72A-83D0-4B18-BE63-0CD0144D427E}"/>

</xml_diff>